<commit_message>
Actualizar ANVEM 2.0 y archivos data
</commit_message>
<xml_diff>
--- a/data/Carlos RamirezT4-2025.xlsx
+++ b/data/Carlos RamirezT4-2025.xlsx
@@ -2,7 +2,6 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
@@ -11,31 +10,44 @@
     <sheet name="By Source" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="###,###,##0"/>
+    <numFmt numFmtId="165" formatCode="###,###,##0.00000000"/>
+    <numFmt numFmtId="166" formatCode="##0.00"/>
+  </numFmts>
+  <fonts count="2">
+    <font>
+      <name val="Calibri"/>
+      <color rgb="FF000000"/>
+      <sz val="11"/>
+    </font>
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
-      <sz val="11"/>
+      <sz val="12"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EEEEEE"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -43,20 +55,44 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -413,134 +449,330 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
+  <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr autoPageBreaks="0" fitToPage="0"/>
   </sheetPr>
-  <dimension ref="D9:I14"/>
+  <dimension ref="C3:I14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
+    <row r="3">
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>ANVEM TUNES</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>RAMIREZ BOJORQUEZ, CARLOS LEONEL (ANVEM TUNES)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>REGALIAS 4TO TRIMESTRE 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Currency : USD</t>
+        </is>
+      </c>
+    </row>
     <row r="9">
-      <c r="D9" s="1" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>SONG</t>
         </is>
       </c>
-      <c r="E9" s="1" t="inlineStr">
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>UNITS</t>
         </is>
       </c>
-      <c r="F9" s="1" t="inlineStr">
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>ROYALTIES</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="D10" s="1" t="inlineStr">
-        <is>
-          <t>quiereme mientras se pueda</t>
-        </is>
-      </c>
-      <c r="E10" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="F10" s="1" t="n">
-        <v>0.001627022494940979</v>
-      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>4526</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>EL JR</t>
+        </is>
+      </c>
+      <c r="E10" s="10" t="n">
+        <v>16523</v>
+      </c>
+      <c r="F10" s="11" t="n">
+        <v>0.24201843</v>
+      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="D11" s="1" t="inlineStr">
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>5061</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>EL INVICTO</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="n">
+        <v>13459</v>
+      </c>
+      <c r="F11" s="11" t="n">
+        <v>0.24031585</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Total Royalties</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>0.6246710300000007</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>5062</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>SOMOS UNO</t>
+        </is>
+      </c>
+      <c r="E12" s="10" t="n">
+        <v>5521</v>
+      </c>
+      <c r="F12" s="11" t="n">
+        <v>0.14233675</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Prior Balance</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>18.36</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Taxes</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>-1.8984671</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="D14" s="6" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E11" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="F11" s="1" t="n">
-        <v>0.001627022</v>
-      </c>
-    </row>
-    <row r="14">
+      <c r="E14" s="10" t="n">
+        <v>35503</v>
+      </c>
+      <c r="F14" s="11" t="n">
+        <v>0.62467103</v>
+      </c>
       <c r="H14" t="inlineStr">
         <is>
           <t>Net Payment</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>0.001627022</v>
+        <v>0.6246710300000007</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" firstPageNumber="0" useFirstPageNumber="0" blackAndWhite="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
+  <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr autoPageBreaks="0" fitToPage="0"/>
   </sheetPr>
-  <dimension ref="D9:I14"/>
+  <dimension ref="C3:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+  </cols>
   <sheetData>
+    <row r="3">
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>ANVEM TUNES</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>RAMIREZ BOJORQUEZ, CARLOS LEONEL (ANVEM TUNES)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>REGALIAS 4TO TRIMESTRE 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Currency : USD</t>
+        </is>
+      </c>
+    </row>
     <row r="9">
-      <c r="D9" s="1" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>SOURCE</t>
         </is>
       </c>
-      <c r="E9" s="1" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>UNITS</t>
         </is>
       </c>
-      <c r="F9" s="1" t="inlineStr">
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>ROYALTIES</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="D10" s="1" t="inlineStr">
-        <is>
-          <t>iTunes Match</t>
-        </is>
-      </c>
-      <c r="E10" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="F10" s="1" t="n">
-        <v>0.001627022494940979</v>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Spotify</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="n">
+        <v>35114</v>
+      </c>
+      <c r="E10" s="11" t="n">
+        <v>0.55302085</v>
       </c>
     </row>
     <row r="11">
-      <c r="D11" s="1" t="inlineStr">
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Apple Music</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="n">
+        <v>232</v>
+      </c>
+      <c r="E11" s="11" t="n">
+        <v>0.04150264</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="D12" s="10" t="n">
+        <v>114</v>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>0.02190847</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>MUSIXMATCH</t>
+        </is>
+      </c>
+      <c r="D13" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="E13" s="11" t="n">
+        <v>0.00478124</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>YouTube (Domestic)</t>
+        </is>
+      </c>
+      <c r="D14" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="E14" s="11" t="n">
+        <v>0.0035</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>amazon</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="E15" s="11" t="n">
+        <v>-4.217e-05</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E11" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="F11" s="1" t="n">
-        <v>0.001627022</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>Net Payment</t>
-        </is>
-      </c>
-      <c r="I14" t="n">
-        <v>0.001627022</v>
+      <c r="D17" s="10" t="n">
+        <v>35503</v>
+      </c>
+      <c r="E17" s="11" t="n">
+        <v>0.62467103</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" firstPageNumber="0" useFirstPageNumber="0" blackAndWhite="0"/>
 </worksheet>
 </file>
</xml_diff>